<commit_message>
chore: demo configs bijgewerkt zonder score_type, rapport module
Demo config bestanden opnieuw gegenereerd met het 4-koloms formaat.
App.py en rapport.py updates uit parallel sessie meegenomen.
</commit_message>
<xml_diff>
--- a/data/demo/biomed_aumc_2026/config.xlsx
+++ b/data/demo/biomed_aumc_2026/config.xlsx
@@ -595,14 +595,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="35" customWidth="1" min="3" max="3"/>
     <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -626,11 +625,6 @@
           <t>criterium (optioneel)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>score_type</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -653,11 +647,6 @@
           <t>Analytisch denken</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>schaalscore</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -680,11 +669,6 @@
           <t>Methodologisch inzicht</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>schaalscore</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -707,11 +691,6 @@
           <t>Analytisch denken</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>schaalscore</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -734,11 +713,6 @@
           <t>Probleemoplossend vermogen</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>schaalscore</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -761,11 +735,6 @@
           <t>Communicatieve vaardigheden</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>schaalscore</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -788,11 +757,6 @@
           <t>Methodologisch inzicht</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>schaalscore</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -816,11 +780,6 @@
           <t>Analytisch denken</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>schaal 1-3</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -844,11 +803,6 @@
           <t>Communicatieve vaardigheden</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>schaal 1-3</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -871,11 +825,6 @@
           <t>Sociale intelligentie</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>schaalscore</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -896,11 +845,6 @@
       <c r="D11" s="4" t="inlineStr">
         <is>
           <t>Wetenschappelijk redeneren</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>schaalscore</t>
         </is>
       </c>
     </row>

</xml_diff>